<commit_message>
Aggiungo tutti i partecipanti
</commit_message>
<xml_diff>
--- a/data/pronostici/TOTOMONDIALE2026_Andrea_Esposito.xlsx
+++ b/data/pronostici/TOTOMONDIALE2026_Andrea_Esposito.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e.castiello\Documents\totomondiale\data\pronostici\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B36E1D0-6B65-4902-B443-8A051DF82F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5E1800-CFFC-4036-A636-9B12875353CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -865,9 +865,6 @@
     <t>Raphinha</t>
   </si>
   <si>
-    <t>Giménez</t>
-  </si>
-  <si>
     <t>Mahrez</t>
   </si>
   <si>
@@ -875,6 +872,9 @@
   </si>
   <si>
     <t>McTominay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jimenez </t>
   </si>
 </sst>
 </file>
@@ -1472,6 +1472,108 @@
     <xf numFmtId="16" fontId="0" fillId="7" borderId="25" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1496,104 +1598,35 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1601,7 +1634,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1621,45 +1660,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2542,273 +2542,247 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="90" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="79"/>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="92"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="80" t="s">
+      <c r="A2" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81" t="s">
+      <c r="B2" s="94"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
+      <c r="E2" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="82"/>
+      <c r="F2" s="95"/>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="84" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="74"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="74" t="s">
+      <c r="B3" s="85"/>
+      <c r="C3" s="85"/>
+      <c r="D3" s="85"/>
+      <c r="E3" s="85" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="75"/>
+      <c r="F3" s="86"/>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="74"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74" t="s">
+      <c r="B4" s="85"/>
+      <c r="C4" s="85"/>
+      <c r="D4" s="85"/>
+      <c r="E4" s="85" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="75"/>
+      <c r="F4" s="86"/>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="76" t="s">
+      <c r="A5" s="84" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="74"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="74"/>
-      <c r="E5" s="74" t="s">
+      <c r="B5" s="85"/>
+      <c r="C5" s="85"/>
+      <c r="D5" s="85"/>
+      <c r="E5" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="75"/>
+      <c r="F5" s="86"/>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="83"/>
-      <c r="B6" s="84"/>
-      <c r="C6" s="84"/>
-      <c r="D6" s="84"/>
-      <c r="E6" s="84"/>
-      <c r="F6" s="85"/>
+      <c r="A6" s="87"/>
+      <c r="B6" s="88"/>
+      <c r="C6" s="88"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="89"/>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="76" t="s">
+      <c r="A7" s="84" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="74"/>
-      <c r="C7" s="74"/>
-      <c r="D7" s="74"/>
-      <c r="E7" s="74" t="s">
+      <c r="B7" s="85"/>
+      <c r="C7" s="85"/>
+      <c r="D7" s="85"/>
+      <c r="E7" s="85" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="75"/>
+      <c r="F7" s="86"/>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="76" t="s">
+      <c r="A8" s="84" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="74"/>
-      <c r="C8" s="74"/>
-      <c r="D8" s="74"/>
-      <c r="E8" s="74" t="s">
+      <c r="B8" s="85"/>
+      <c r="C8" s="85"/>
+      <c r="D8" s="85"/>
+      <c r="E8" s="85" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="75"/>
+      <c r="F8" s="86"/>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="76" t="s">
+      <c r="A9" s="84" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="74"/>
-      <c r="C9" s="74"/>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74" t="s">
+      <c r="B9" s="85"/>
+      <c r="C9" s="85"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="75"/>
+      <c r="F9" s="86"/>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="83"/>
-      <c r="B10" s="84"/>
-      <c r="C10" s="84"/>
-      <c r="D10" s="84"/>
-      <c r="E10" s="84"/>
-      <c r="F10" s="85"/>
+      <c r="A10" s="87"/>
+      <c r="B10" s="88"/>
+      <c r="C10" s="88"/>
+      <c r="D10" s="88"/>
+      <c r="E10" s="88"/>
+      <c r="F10" s="89"/>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="76" t="s">
+      <c r="A11" s="84" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="74"/>
-      <c r="C11" s="74"/>
-      <c r="D11" s="74"/>
-      <c r="E11" s="74" t="s">
+      <c r="B11" s="85"/>
+      <c r="C11" s="85"/>
+      <c r="D11" s="85"/>
+      <c r="E11" s="85" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="75"/>
+      <c r="F11" s="86"/>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="76" t="s">
+      <c r="A12" s="84" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="74"/>
-      <c r="C12" s="74"/>
-      <c r="D12" s="74"/>
-      <c r="E12" s="74" t="s">
+      <c r="B12" s="85"/>
+      <c r="C12" s="85"/>
+      <c r="D12" s="85"/>
+      <c r="E12" s="85" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="75"/>
+      <c r="F12" s="86"/>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="76" t="s">
+      <c r="A13" s="84" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="74"/>
-      <c r="C13" s="74"/>
-      <c r="D13" s="74"/>
-      <c r="E13" s="74" t="s">
+      <c r="B13" s="85"/>
+      <c r="C13" s="85"/>
+      <c r="D13" s="85"/>
+      <c r="E13" s="85" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="75"/>
+      <c r="F13" s="86"/>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="83"/>
-      <c r="B14" s="84"/>
-      <c r="C14" s="84"/>
-      <c r="D14" s="84"/>
-      <c r="E14" s="84"/>
-      <c r="F14" s="85"/>
+      <c r="A14" s="87"/>
+      <c r="B14" s="88"/>
+      <c r="C14" s="88"/>
+      <c r="D14" s="88"/>
+      <c r="E14" s="88"/>
+      <c r="F14" s="89"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="76" t="s">
+      <c r="A15" s="84" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="74"/>
-      <c r="C15" s="74"/>
-      <c r="D15" s="74"/>
-      <c r="E15" s="74" t="s">
+      <c r="B15" s="85"/>
+      <c r="C15" s="85"/>
+      <c r="D15" s="85"/>
+      <c r="E15" s="85" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="75"/>
+      <c r="F15" s="86"/>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="76" t="s">
+      <c r="A16" s="84" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="74"/>
-      <c r="C16" s="74"/>
-      <c r="D16" s="74"/>
-      <c r="E16" s="74" t="s">
+      <c r="B16" s="85"/>
+      <c r="C16" s="85"/>
+      <c r="D16" s="85"/>
+      <c r="E16" s="85" t="s">
         <v>22</v>
       </c>
-      <c r="F16" s="75"/>
+      <c r="F16" s="86"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="76" t="s">
+      <c r="A17" s="84" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="74"/>
-      <c r="C17" s="74"/>
-      <c r="D17" s="74"/>
-      <c r="E17" s="74" t="s">
+      <c r="B17" s="85"/>
+      <c r="C17" s="85"/>
+      <c r="D17" s="85"/>
+      <c r="E17" s="85" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="75"/>
+      <c r="F17" s="86"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="76" t="s">
+      <c r="A18" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="74"/>
-      <c r="C18" s="74"/>
-      <c r="D18" s="74"/>
-      <c r="E18" s="74" t="s">
+      <c r="B18" s="85"/>
+      <c r="C18" s="85"/>
+      <c r="D18" s="85"/>
+      <c r="E18" s="85" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="75"/>
+      <c r="F18" s="86"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="76" t="s">
+      <c r="A19" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="74"/>
-      <c r="C19" s="74"/>
-      <c r="D19" s="74"/>
-      <c r="E19" s="74" t="s">
+      <c r="B19" s="85"/>
+      <c r="C19" s="85"/>
+      <c r="D19" s="85"/>
+      <c r="E19" s="85" t="s">
         <v>15</v>
       </c>
-      <c r="F19" s="75"/>
+      <c r="F19" s="86"/>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="86" t="s">
+      <c r="A20" s="75" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="87"/>
-      <c r="C20" s="87"/>
-      <c r="D20" s="87"/>
-      <c r="E20" s="87"/>
-      <c r="F20" s="88"/>
+      <c r="B20" s="76"/>
+      <c r="C20" s="76"/>
+      <c r="D20" s="76"/>
+      <c r="E20" s="76"/>
+      <c r="F20" s="77"/>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="89"/>
-      <c r="B21" s="90"/>
-      <c r="C21" s="90"/>
-      <c r="D21" s="90"/>
-      <c r="E21" s="90"/>
-      <c r="F21" s="91"/>
+      <c r="A21" s="78"/>
+      <c r="B21" s="79"/>
+      <c r="C21" s="79"/>
+      <c r="D21" s="79"/>
+      <c r="E21" s="79"/>
+      <c r="F21" s="80"/>
     </row>
     <row r="22" spans="1:6" ht="14.5" thickBot="1">
-      <c r="A22" s="92"/>
-      <c r="B22" s="93"/>
-      <c r="C22" s="93"/>
-      <c r="D22" s="93"/>
-      <c r="E22" s="93"/>
-      <c r="F22" s="94"/>
+      <c r="A22" s="81"/>
+      <c r="B22" s="82"/>
+      <c r="C22" s="82"/>
+      <c r="D22" s="82"/>
+      <c r="E22" s="82"/>
+      <c r="F22" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="A20:F22"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A9:D9"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A4:D4"/>
@@ -2818,6 +2792,32 @@
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="A20:F22"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="E19:F19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2840,97 +2840,97 @@
   <sheetData>
     <row r="1" spans="1:20" ht="16.5" customHeight="1"/>
     <row r="2" spans="1:20">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="70" t="s">
+      <c r="B2" s="43"/>
+      <c r="C2" s="44" t="s">
         <v>269</v>
       </c>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="69"/>
-      <c r="C3" s="70" t="s">
+      <c r="B3" s="43"/>
+      <c r="C3" s="44" t="s">
         <v>270</v>
       </c>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
-      <c r="F3" s="70"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
     </row>
     <row r="5" spans="1:20">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="33"/>
-      <c r="I5" s="33"/>
-      <c r="J5" s="33"/>
-      <c r="K5" s="33"/>
-      <c r="L5" s="33"/>
-      <c r="M5" s="33"/>
-      <c r="N5" s="33"/>
-      <c r="O5" s="33"/>
-      <c r="P5" s="33"/>
-      <c r="Q5" s="33"/>
-      <c r="R5" s="33"/>
-      <c r="S5" s="33"/>
-      <c r="T5" s="33"/>
+      <c r="B5" s="67"/>
+      <c r="C5" s="67"/>
+      <c r="D5" s="67"/>
+      <c r="E5" s="67"/>
+      <c r="F5" s="67"/>
+      <c r="G5" s="67"/>
+      <c r="H5" s="67"/>
+      <c r="I5" s="67"/>
+      <c r="J5" s="67"/>
+      <c r="K5" s="67"/>
+      <c r="L5" s="67"/>
+      <c r="M5" s="67"/>
+      <c r="N5" s="67"/>
+      <c r="O5" s="67"/>
+      <c r="P5" s="67"/>
+      <c r="Q5" s="67"/>
+      <c r="R5" s="67"/>
+      <c r="S5" s="67"/>
+      <c r="T5" s="67"/>
     </row>
     <row r="6" spans="1:20" ht="15" thickBot="1">
-      <c r="A6" s="33"/>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="33"/>
-      <c r="K6" s="33"/>
-      <c r="L6" s="33"/>
-      <c r="M6" s="33"/>
-      <c r="N6" s="33"/>
-      <c r="O6" s="33"/>
-      <c r="P6" s="33"/>
-      <c r="Q6" s="33"/>
-      <c r="R6" s="33"/>
-      <c r="S6" s="33"/>
-      <c r="T6" s="33"/>
+      <c r="A6" s="67"/>
+      <c r="B6" s="67"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="67"/>
+      <c r="G6" s="67"/>
+      <c r="H6" s="67"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="67"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="67"/>
+      <c r="M6" s="67"/>
+      <c r="N6" s="67"/>
+      <c r="O6" s="67"/>
+      <c r="P6" s="67"/>
+      <c r="Q6" s="67"/>
+      <c r="R6" s="67"/>
+      <c r="S6" s="67"/>
+      <c r="T6" s="67"/>
     </row>
     <row r="7" spans="1:20" ht="16.5" customHeight="1">
-      <c r="A7" s="38" t="s">
+      <c r="A7" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="39"/>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
-      <c r="G7" s="39"/>
-      <c r="H7" s="40"/>
+      <c r="B7" s="73"/>
+      <c r="C7" s="73"/>
+      <c r="D7" s="73"/>
+      <c r="E7" s="73"/>
+      <c r="F7" s="73"/>
+      <c r="G7" s="73"/>
+      <c r="H7" s="74"/>
       <c r="I7" s="1"/>
-      <c r="J7" s="38" t="s">
+      <c r="J7" s="72" t="s">
         <v>31</v>
       </c>
-      <c r="K7" s="39"/>
-      <c r="L7" s="39"/>
-      <c r="M7" s="39"/>
-      <c r="N7" s="39"/>
-      <c r="O7" s="39"/>
-      <c r="P7" s="39"/>
-      <c r="Q7" s="40"/>
+      <c r="K7" s="73"/>
+      <c r="L7" s="73"/>
+      <c r="M7" s="73"/>
+      <c r="N7" s="73"/>
+      <c r="O7" s="73"/>
+      <c r="P7" s="73"/>
+      <c r="Q7" s="74"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
       <c r="T7" s="1"/>
@@ -2942,11 +2942,11 @@
       <c r="B8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="68"/>
       <c r="F8" s="4" t="s">
         <v>35</v>
       </c>
@@ -2956,16 +2956,16 @@
       <c r="H8" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="J8" s="35" t="s">
+      <c r="J8" s="69" t="s">
         <v>37</v>
       </c>
-      <c r="K8" s="36"/>
-      <c r="L8" s="36"/>
-      <c r="M8" s="36"/>
-      <c r="N8" s="36"/>
-      <c r="O8" s="36"/>
-      <c r="P8" s="36"/>
-      <c r="Q8" s="37"/>
+      <c r="K8" s="70"/>
+      <c r="L8" s="70"/>
+      <c r="M8" s="70"/>
+      <c r="N8" s="70"/>
+      <c r="O8" s="70"/>
+      <c r="P8" s="70"/>
+      <c r="Q8" s="71"/>
     </row>
     <row r="9" spans="1:20" ht="18.5">
       <c r="A9" s="17">
@@ -2974,11 +2974,11 @@
       <c r="B9" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="45" t="s">
+      <c r="C9" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="46"/>
-      <c r="E9" s="47"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="36"/>
       <c r="F9" s="7">
         <v>1</v>
       </c>
@@ -2988,20 +2988,20 @@
       <c r="H9" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="J9" s="35" t="s">
+      <c r="J9" s="69" t="s">
         <v>40</v>
       </c>
-      <c r="K9" s="36"/>
-      <c r="L9" s="36" t="s">
+      <c r="K9" s="70"/>
+      <c r="L9" s="70" t="s">
         <v>41</v>
       </c>
-      <c r="M9" s="36"/>
-      <c r="N9" s="36"/>
-      <c r="O9" s="36" t="s">
+      <c r="M9" s="70"/>
+      <c r="N9" s="70"/>
+      <c r="O9" s="70" t="s">
         <v>42</v>
       </c>
-      <c r="P9" s="36"/>
-      <c r="Q9" s="37"/>
+      <c r="P9" s="70"/>
+      <c r="Q9" s="71"/>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" s="19">
@@ -3010,11 +3010,11 @@
       <c r="B10" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="48" t="s">
+      <c r="C10" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="49"/>
-      <c r="E10" s="50"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="39"/>
       <c r="F10" s="9">
         <v>1</v>
       </c>
@@ -3024,20 +3024,20 @@
       <c r="H10" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="J10" s="41" t="s">
+      <c r="J10" s="63" t="s">
         <v>38</v>
       </c>
-      <c r="K10" s="42"/>
-      <c r="L10" s="43" t="s">
+      <c r="K10" s="65"/>
+      <c r="L10" s="46" t="s">
         <v>171</v>
       </c>
-      <c r="M10" s="43"/>
-      <c r="N10" s="43"/>
-      <c r="O10" s="43" t="s">
+      <c r="M10" s="46"/>
+      <c r="N10" s="46"/>
+      <c r="O10" s="46" t="s">
         <v>170</v>
       </c>
-      <c r="P10" s="43"/>
-      <c r="Q10" s="44"/>
+      <c r="P10" s="46"/>
+      <c r="Q10" s="47"/>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" s="19">
@@ -3046,11 +3046,11 @@
       <c r="B11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="49"/>
-      <c r="E11" s="50"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="39"/>
       <c r="F11" s="9" t="s">
         <v>196</v>
       </c>
@@ -3060,20 +3060,20 @@
       <c r="H11" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="J11" s="41" t="s">
+      <c r="J11" s="63" t="s">
         <v>44</v>
       </c>
-      <c r="K11" s="42"/>
-      <c r="L11" s="43" t="s">
+      <c r="K11" s="65"/>
+      <c r="L11" s="46" t="s">
         <v>174</v>
       </c>
-      <c r="M11" s="43"/>
-      <c r="N11" s="43"/>
-      <c r="O11" s="43" t="s">
+      <c r="M11" s="46"/>
+      <c r="N11" s="46"/>
+      <c r="O11" s="46" t="s">
         <v>136</v>
       </c>
-      <c r="P11" s="43"/>
-      <c r="Q11" s="44"/>
+      <c r="P11" s="46"/>
+      <c r="Q11" s="47"/>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" s="17">
@@ -3082,11 +3082,11 @@
       <c r="B12" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="45" t="s">
+      <c r="C12" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="46"/>
-      <c r="E12" s="47"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="36"/>
       <c r="F12" s="7">
         <v>1</v>
       </c>
@@ -3096,20 +3096,20 @@
       <c r="H12" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="J12" s="41" t="s">
+      <c r="J12" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="K12" s="42"/>
-      <c r="L12" s="43" t="s">
+      <c r="K12" s="65"/>
+      <c r="L12" s="46" t="s">
         <v>139</v>
       </c>
-      <c r="M12" s="43"/>
-      <c r="N12" s="43"/>
-      <c r="O12" s="43" t="s">
+      <c r="M12" s="46"/>
+      <c r="N12" s="46"/>
+      <c r="O12" s="46" t="s">
         <v>175</v>
       </c>
-      <c r="P12" s="43"/>
-      <c r="Q12" s="44"/>
+      <c r="P12" s="46"/>
+      <c r="Q12" s="47"/>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" s="17">
@@ -3118,11 +3118,11 @@
       <c r="B13" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="45" t="s">
+      <c r="C13" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="D13" s="46"/>
-      <c r="E13" s="47"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="36"/>
       <c r="F13" s="7">
         <v>2</v>
       </c>
@@ -3132,20 +3132,20 @@
       <c r="H13" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="J13" s="41" t="s">
+      <c r="J13" s="63" t="s">
         <v>46</v>
       </c>
-      <c r="K13" s="42"/>
-      <c r="L13" s="43" t="s">
+      <c r="K13" s="65"/>
+      <c r="L13" s="46" t="s">
         <v>177</v>
       </c>
-      <c r="M13" s="43"/>
-      <c r="N13" s="43"/>
-      <c r="O13" s="43" t="s">
+      <c r="M13" s="46"/>
+      <c r="N13" s="46"/>
+      <c r="O13" s="46" t="s">
         <v>142</v>
       </c>
-      <c r="P13" s="43"/>
-      <c r="Q13" s="44"/>
+      <c r="P13" s="46"/>
+      <c r="Q13" s="47"/>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" s="19">
@@ -3154,11 +3154,11 @@
       <c r="B14" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="48" t="s">
+      <c r="C14" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="49"/>
-      <c r="E14" s="50"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="39"/>
       <c r="F14" s="9">
         <v>1</v>
       </c>
@@ -3168,20 +3168,20 @@
       <c r="H14" s="20" t="s">
         <v>272</v>
       </c>
-      <c r="J14" s="41" t="s">
+      <c r="J14" s="63" t="s">
         <v>51</v>
       </c>
-      <c r="K14" s="42"/>
-      <c r="L14" s="43" t="s">
+      <c r="K14" s="65"/>
+      <c r="L14" s="46" t="s">
         <v>179</v>
       </c>
-      <c r="M14" s="43"/>
-      <c r="N14" s="43"/>
-      <c r="O14" s="43" t="s">
+      <c r="M14" s="46"/>
+      <c r="N14" s="46"/>
+      <c r="O14" s="46" t="s">
         <v>178</v>
       </c>
-      <c r="P14" s="43"/>
-      <c r="Q14" s="44"/>
+      <c r="P14" s="46"/>
+      <c r="Q14" s="47"/>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" s="19">
@@ -3190,11 +3190,11 @@
       <c r="B15" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="48" t="s">
+      <c r="C15" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="D15" s="49"/>
-      <c r="E15" s="50"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="39"/>
       <c r="F15" s="9">
         <v>2</v>
       </c>
@@ -3202,22 +3202,22 @@
         <v>198</v>
       </c>
       <c r="H15" s="20" t="s">
-        <v>276</v>
-      </c>
-      <c r="J15" s="41" t="s">
+        <v>275</v>
+      </c>
+      <c r="J15" s="63" t="s">
         <v>53</v>
       </c>
-      <c r="K15" s="42"/>
-      <c r="L15" s="43" t="s">
+      <c r="K15" s="65"/>
+      <c r="L15" s="46" t="s">
         <v>181</v>
       </c>
-      <c r="M15" s="43"/>
-      <c r="N15" s="43"/>
-      <c r="O15" s="43" t="s">
+      <c r="M15" s="46"/>
+      <c r="N15" s="46"/>
+      <c r="O15" s="46" t="s">
         <v>180</v>
       </c>
-      <c r="P15" s="43"/>
-      <c r="Q15" s="44"/>
+      <c r="P15" s="46"/>
+      <c r="Q15" s="47"/>
     </row>
     <row r="16" spans="1:20">
       <c r="A16" s="19">
@@ -3226,11 +3226,11 @@
       <c r="B16" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="48" t="s">
+      <c r="C16" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="49"/>
-      <c r="E16" s="50"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="39"/>
       <c r="F16" s="9">
         <v>2</v>
       </c>
@@ -3240,20 +3240,20 @@
       <c r="H16" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="J16" s="41" t="s">
+      <c r="J16" s="63" t="s">
         <v>55</v>
       </c>
-      <c r="K16" s="42"/>
-      <c r="L16" s="43" t="s">
+      <c r="K16" s="65"/>
+      <c r="L16" s="46" t="s">
         <v>183</v>
       </c>
-      <c r="M16" s="43"/>
-      <c r="N16" s="43"/>
-      <c r="O16" s="43" t="s">
+      <c r="M16" s="46"/>
+      <c r="N16" s="46"/>
+      <c r="O16" s="46" t="s">
         <v>184</v>
       </c>
-      <c r="P16" s="43"/>
-      <c r="Q16" s="44"/>
+      <c r="P16" s="46"/>
+      <c r="Q16" s="47"/>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="19">
@@ -3262,11 +3262,11 @@
       <c r="B17" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="49"/>
-      <c r="E17" s="50"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="39"/>
       <c r="F17" s="9">
         <v>1</v>
       </c>
@@ -3276,20 +3276,20 @@
       <c r="H17" s="20" t="s">
         <v>226</v>
       </c>
-      <c r="J17" s="41" t="s">
+      <c r="J17" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="K17" s="42"/>
-      <c r="L17" s="43" t="s">
+      <c r="K17" s="65"/>
+      <c r="L17" s="46" t="s">
         <v>152</v>
       </c>
-      <c r="M17" s="43"/>
-      <c r="N17" s="43"/>
-      <c r="O17" s="43" t="s">
+      <c r="M17" s="46"/>
+      <c r="N17" s="46"/>
+      <c r="O17" s="46" t="s">
         <v>188</v>
       </c>
-      <c r="P17" s="43"/>
-      <c r="Q17" s="44"/>
+      <c r="P17" s="46"/>
+      <c r="Q17" s="47"/>
     </row>
     <row r="18" spans="1:17">
       <c r="A18" s="19">
@@ -3298,11 +3298,11 @@
       <c r="B18" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="48" t="s">
+      <c r="C18" s="37" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="49"/>
-      <c r="E18" s="50"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="39"/>
       <c r="F18" s="9">
         <v>1</v>
       </c>
@@ -3312,20 +3312,20 @@
       <c r="H18" s="20" t="s">
         <v>227</v>
       </c>
-      <c r="J18" s="41" t="s">
+      <c r="J18" s="63" t="s">
         <v>59</v>
       </c>
-      <c r="K18" s="42"/>
-      <c r="L18" s="43" t="s">
+      <c r="K18" s="65"/>
+      <c r="L18" s="46" t="s">
         <v>190</v>
       </c>
-      <c r="M18" s="43"/>
-      <c r="N18" s="43"/>
-      <c r="O18" s="43" t="s">
+      <c r="M18" s="46"/>
+      <c r="N18" s="46"/>
+      <c r="O18" s="46" t="s">
         <v>191</v>
       </c>
-      <c r="P18" s="43"/>
-      <c r="Q18" s="44"/>
+      <c r="P18" s="46"/>
+      <c r="Q18" s="47"/>
     </row>
     <row r="19" spans="1:17">
       <c r="A19" s="17">
@@ -3334,11 +3334,11 @@
       <c r="B19" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="45" t="s">
+      <c r="C19" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="D19" s="46"/>
-      <c r="E19" s="47"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="36"/>
       <c r="F19" s="7">
         <v>1</v>
       </c>
@@ -3348,20 +3348,20 @@
       <c r="H19" s="18" t="s">
         <v>228</v>
       </c>
-      <c r="J19" s="41" t="s">
+      <c r="J19" s="63" t="s">
         <v>61</v>
       </c>
-      <c r="K19" s="42"/>
-      <c r="L19" s="43" t="s">
+      <c r="K19" s="65"/>
+      <c r="L19" s="46" t="s">
         <v>157</v>
       </c>
-      <c r="M19" s="43"/>
-      <c r="N19" s="43"/>
-      <c r="O19" s="43" t="s">
+      <c r="M19" s="46"/>
+      <c r="N19" s="46"/>
+      <c r="O19" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="P19" s="43"/>
-      <c r="Q19" s="44"/>
+      <c r="P19" s="46"/>
+      <c r="Q19" s="47"/>
     </row>
     <row r="20" spans="1:17">
       <c r="A20" s="17">
@@ -3370,11 +3370,11 @@
       <c r="B20" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="45" t="s">
+      <c r="C20" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="D20" s="46"/>
-      <c r="E20" s="47"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="36"/>
       <c r="F20" s="7">
         <v>1</v>
       </c>
@@ -3384,20 +3384,20 @@
       <c r="H20" s="18" t="s">
         <v>229</v>
       </c>
-      <c r="J20" s="41" t="s">
+      <c r="J20" s="63" t="s">
         <v>63</v>
       </c>
-      <c r="K20" s="42"/>
-      <c r="L20" s="43" t="s">
+      <c r="K20" s="65"/>
+      <c r="L20" s="46" t="s">
         <v>163</v>
       </c>
-      <c r="M20" s="43"/>
-      <c r="N20" s="43"/>
-      <c r="O20" s="43" t="s">
+      <c r="M20" s="46"/>
+      <c r="N20" s="46"/>
+      <c r="O20" s="46" t="s">
         <v>193</v>
       </c>
-      <c r="P20" s="43"/>
-      <c r="Q20" s="44"/>
+      <c r="P20" s="46"/>
+      <c r="Q20" s="47"/>
     </row>
     <row r="21" spans="1:17" ht="15" thickBot="1">
       <c r="A21" s="17">
@@ -3406,11 +3406,11 @@
       <c r="B21" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="45" t="s">
+      <c r="C21" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="D21" s="46"/>
-      <c r="E21" s="47"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="36"/>
       <c r="F21" s="7">
         <v>1</v>
       </c>
@@ -3420,20 +3420,20 @@
       <c r="H21" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="J21" s="53" t="s">
+      <c r="J21" s="64" t="s">
         <v>65</v>
       </c>
-      <c r="K21" s="54"/>
-      <c r="L21" s="51" t="s">
+      <c r="K21" s="66"/>
+      <c r="L21" s="49" t="s">
         <v>195</v>
       </c>
-      <c r="M21" s="51"/>
-      <c r="N21" s="51"/>
-      <c r="O21" s="51" t="s">
+      <c r="M21" s="49"/>
+      <c r="N21" s="49"/>
+      <c r="O21" s="49" t="s">
         <v>194</v>
       </c>
-      <c r="P21" s="51"/>
-      <c r="Q21" s="52"/>
+      <c r="P21" s="49"/>
+      <c r="Q21" s="50"/>
     </row>
     <row r="22" spans="1:17" ht="15" thickBot="1">
       <c r="A22" s="17">
@@ -3442,11 +3442,11 @@
       <c r="B22" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C22" s="45" t="s">
+      <c r="C22" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="D22" s="46"/>
-      <c r="E22" s="47"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="36"/>
       <c r="F22" s="7">
         <v>1</v>
       </c>
@@ -3464,11 +3464,11 @@
       <c r="B23" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C23" s="48" t="s">
+      <c r="C23" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="D23" s="49"/>
-      <c r="E23" s="50"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="39"/>
       <c r="F23" s="9">
         <v>2</v>
       </c>
@@ -3478,13 +3478,13 @@
       <c r="H23" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="L23" s="55" t="s">
+      <c r="L23" s="51" t="s">
         <v>68</v>
       </c>
-      <c r="M23" s="56"/>
-      <c r="N23" s="56"/>
-      <c r="O23" s="56"/>
-      <c r="P23" s="57"/>
+      <c r="M23" s="52"/>
+      <c r="N23" s="52"/>
+      <c r="O23" s="52"/>
+      <c r="P23" s="53"/>
     </row>
     <row r="24" spans="1:17">
       <c r="A24" s="19">
@@ -3493,11 +3493,11 @@
       <c r="B24" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C24" s="48" t="s">
+      <c r="C24" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="D24" s="49"/>
-      <c r="E24" s="50"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="39"/>
       <c r="F24" s="9" t="s">
         <v>196</v>
       </c>
@@ -3507,13 +3507,13 @@
       <c r="H24" s="20" t="s">
         <v>233</v>
       </c>
-      <c r="L24" s="58" t="s">
+      <c r="L24" s="45" t="s">
         <v>267</v>
       </c>
-      <c r="M24" s="43"/>
-      <c r="N24" s="43"/>
-      <c r="O24" s="43"/>
-      <c r="P24" s="44"/>
+      <c r="M24" s="46"/>
+      <c r="N24" s="46"/>
+      <c r="O24" s="46"/>
+      <c r="P24" s="47"/>
     </row>
     <row r="25" spans="1:17" ht="15" thickBot="1">
       <c r="A25" s="19">
@@ -3522,11 +3522,11 @@
       <c r="B25" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C25" s="48" t="s">
+      <c r="C25" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="D25" s="49"/>
-      <c r="E25" s="50"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="39"/>
       <c r="F25" s="9" t="s">
         <v>196</v>
       </c>
@@ -3536,11 +3536,11 @@
       <c r="H25" s="20" t="s">
         <v>234</v>
       </c>
-      <c r="L25" s="59"/>
-      <c r="M25" s="51"/>
-      <c r="N25" s="51"/>
-      <c r="O25" s="51"/>
-      <c r="P25" s="52"/>
+      <c r="L25" s="48"/>
+      <c r="M25" s="49"/>
+      <c r="N25" s="49"/>
+      <c r="O25" s="49"/>
+      <c r="P25" s="50"/>
     </row>
     <row r="26" spans="1:17" ht="15" thickBot="1">
       <c r="A26" s="17">
@@ -3549,11 +3549,11 @@
       <c r="B26" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="45" t="s">
+      <c r="C26" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="D26" s="46"/>
-      <c r="E26" s="47"/>
+      <c r="D26" s="35"/>
+      <c r="E26" s="36"/>
       <c r="F26" s="7">
         <v>2</v>
       </c>
@@ -3571,11 +3571,11 @@
       <c r="B27" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="45" t="s">
+      <c r="C27" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="D27" s="46"/>
-      <c r="E27" s="47"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="36"/>
       <c r="F27" s="7">
         <v>1</v>
       </c>
@@ -3600,11 +3600,11 @@
       <c r="B28" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C28" s="45" t="s">
+      <c r="C28" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="D28" s="46"/>
-      <c r="E28" s="47"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="36"/>
       <c r="F28" s="7">
         <v>1</v>
       </c>
@@ -3614,15 +3614,15 @@
       <c r="H28" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="L28" s="41" t="s">
+      <c r="L28" s="63" t="s">
         <v>75</v>
       </c>
-      <c r="M28" s="43" t="s">
+      <c r="M28" s="46" t="s">
         <v>267</v>
       </c>
-      <c r="N28" s="43"/>
-      <c r="O28" s="43"/>
-      <c r="P28" s="44"/>
+      <c r="N28" s="46"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="47"/>
     </row>
     <row r="29" spans="1:17">
       <c r="A29" s="17">
@@ -3631,11 +3631,11 @@
       <c r="B29" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="45" t="s">
+      <c r="C29" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="D29" s="46"/>
-      <c r="E29" s="47"/>
+      <c r="D29" s="35"/>
+      <c r="E29" s="36"/>
       <c r="F29" s="7">
         <v>1</v>
       </c>
@@ -3645,11 +3645,11 @@
       <c r="H29" s="18" t="s">
         <v>238</v>
       </c>
-      <c r="L29" s="41"/>
-      <c r="M29" s="43"/>
-      <c r="N29" s="43"/>
-      <c r="O29" s="43"/>
-      <c r="P29" s="44"/>
+      <c r="L29" s="63"/>
+      <c r="M29" s="46"/>
+      <c r="N29" s="46"/>
+      <c r="O29" s="46"/>
+      <c r="P29" s="47"/>
     </row>
     <row r="30" spans="1:17">
       <c r="A30" s="17">
@@ -3658,11 +3658,11 @@
       <c r="B30" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C30" s="45" t="s">
+      <c r="C30" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="D30" s="46"/>
-      <c r="E30" s="47"/>
+      <c r="D30" s="35"/>
+      <c r="E30" s="36"/>
       <c r="F30" s="7">
         <v>1</v>
       </c>
@@ -3672,15 +3672,15 @@
       <c r="H30" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="L30" s="41" t="s">
+      <c r="L30" s="63" t="s">
         <v>78</v>
       </c>
-      <c r="M30" s="43" t="s">
+      <c r="M30" s="46" t="s">
         <v>268</v>
       </c>
-      <c r="N30" s="43"/>
-      <c r="O30" s="43"/>
-      <c r="P30" s="44"/>
+      <c r="N30" s="46"/>
+      <c r="O30" s="46"/>
+      <c r="P30" s="47"/>
     </row>
     <row r="31" spans="1:17" ht="15" thickBot="1">
       <c r="A31" s="19">
@@ -3689,11 +3689,11 @@
       <c r="B31" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C31" s="48" t="s">
+      <c r="C31" s="37" t="s">
         <v>79</v>
       </c>
-      <c r="D31" s="49"/>
-      <c r="E31" s="50"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="39"/>
       <c r="F31" s="9">
         <v>1</v>
       </c>
@@ -3703,11 +3703,11 @@
       <c r="H31" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="L31" s="53"/>
-      <c r="M31" s="51"/>
-      <c r="N31" s="51"/>
-      <c r="O31" s="51"/>
-      <c r="P31" s="52"/>
+      <c r="L31" s="64"/>
+      <c r="M31" s="49"/>
+      <c r="N31" s="49"/>
+      <c r="O31" s="49"/>
+      <c r="P31" s="50"/>
     </row>
     <row r="32" spans="1:17" ht="15" thickBot="1">
       <c r="A32" s="19">
@@ -3716,11 +3716,11 @@
       <c r="B32" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C32" s="48" t="s">
+      <c r="C32" s="37" t="s">
         <v>80</v>
       </c>
-      <c r="D32" s="49"/>
-      <c r="E32" s="50"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="39"/>
       <c r="F32" s="9">
         <v>2</v>
       </c>
@@ -3732,21 +3732,21 @@
       </c>
     </row>
     <row r="33" spans="1:16" ht="18.5">
-      <c r="A33" s="63"/>
-      <c r="B33" s="64"/>
-      <c r="C33" s="64"/>
-      <c r="D33" s="64"/>
-      <c r="E33" s="64"/>
-      <c r="F33" s="64"/>
-      <c r="G33" s="64"/>
-      <c r="H33" s="65"/>
-      <c r="L33" s="55" t="s">
+      <c r="A33" s="57"/>
+      <c r="B33" s="58"/>
+      <c r="C33" s="58"/>
+      <c r="D33" s="58"/>
+      <c r="E33" s="58"/>
+      <c r="F33" s="58"/>
+      <c r="G33" s="58"/>
+      <c r="H33" s="59"/>
+      <c r="L33" s="51" t="s">
         <v>81</v>
       </c>
-      <c r="M33" s="56"/>
-      <c r="N33" s="56"/>
-      <c r="O33" s="56"/>
-      <c r="P33" s="57"/>
+      <c r="M33" s="52"/>
+      <c r="N33" s="52"/>
+      <c r="O33" s="52"/>
+      <c r="P33" s="53"/>
     </row>
     <row r="34" spans="1:16">
       <c r="A34" s="19">
@@ -3755,11 +3755,11 @@
       <c r="B34" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="48" t="s">
+      <c r="C34" s="37" t="s">
         <v>82</v>
       </c>
-      <c r="D34" s="49"/>
-      <c r="E34" s="50"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="39"/>
       <c r="F34" s="9">
         <v>1</v>
       </c>
@@ -3769,13 +3769,13 @@
       <c r="H34" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="L34" s="58" t="s">
+      <c r="L34" s="45" t="s">
         <v>249</v>
       </c>
-      <c r="M34" s="43"/>
-      <c r="N34" s="43"/>
-      <c r="O34" s="43"/>
-      <c r="P34" s="44"/>
+      <c r="M34" s="46"/>
+      <c r="N34" s="46"/>
+      <c r="O34" s="46"/>
+      <c r="P34" s="47"/>
     </row>
     <row r="35" spans="1:16" ht="15" thickBot="1">
       <c r="A35" s="19">
@@ -3784,11 +3784,11 @@
       <c r="B35" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C35" s="48" t="s">
+      <c r="C35" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="D35" s="49"/>
-      <c r="E35" s="50"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="39"/>
       <c r="F35" s="9">
         <v>1</v>
       </c>
@@ -3798,11 +3798,11 @@
       <c r="H35" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="L35" s="59"/>
-      <c r="M35" s="51"/>
-      <c r="N35" s="51"/>
-      <c r="O35" s="51"/>
-      <c r="P35" s="52"/>
+      <c r="L35" s="48"/>
+      <c r="M35" s="49"/>
+      <c r="N35" s="49"/>
+      <c r="O35" s="49"/>
+      <c r="P35" s="50"/>
     </row>
     <row r="36" spans="1:16" ht="15" thickBot="1">
       <c r="A36" s="17">
@@ -3811,11 +3811,11 @@
       <c r="B36" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C36" s="45" t="s">
+      <c r="C36" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="D36" s="46"/>
-      <c r="E36" s="47"/>
+      <c r="D36" s="35"/>
+      <c r="E36" s="36"/>
       <c r="F36" s="7">
         <v>1</v>
       </c>
@@ -3833,11 +3833,11 @@
       <c r="B37" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C37" s="45" t="s">
+      <c r="C37" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="D37" s="46"/>
-      <c r="E37" s="47"/>
+      <c r="D37" s="35"/>
+      <c r="E37" s="36"/>
       <c r="F37" s="7">
         <v>1</v>
       </c>
@@ -3845,15 +3845,15 @@
         <v>197</v>
       </c>
       <c r="H37" s="18" t="s">
-        <v>273</v>
-      </c>
-      <c r="L37" s="55" t="s">
+        <v>276</v>
+      </c>
+      <c r="L37" s="51" t="s">
         <v>86</v>
       </c>
-      <c r="M37" s="56"/>
-      <c r="N37" s="56"/>
-      <c r="O37" s="56"/>
-      <c r="P37" s="57"/>
+      <c r="M37" s="52"/>
+      <c r="N37" s="52"/>
+      <c r="O37" s="52"/>
+      <c r="P37" s="53"/>
     </row>
     <row r="38" spans="1:16">
       <c r="A38" s="17">
@@ -3862,11 +3862,11 @@
       <c r="B38" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C38" s="45" t="s">
+      <c r="C38" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="D38" s="46"/>
-      <c r="E38" s="47"/>
+      <c r="D38" s="35"/>
+      <c r="E38" s="36"/>
       <c r="F38" s="7">
         <v>1</v>
       </c>
@@ -3876,13 +3876,13 @@
       <c r="H38" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="L38" s="58" t="s">
+      <c r="L38" s="45" t="s">
         <v>236</v>
       </c>
-      <c r="M38" s="43"/>
-      <c r="N38" s="43"/>
-      <c r="O38" s="43"/>
-      <c r="P38" s="44"/>
+      <c r="M38" s="46"/>
+      <c r="N38" s="46"/>
+      <c r="O38" s="46"/>
+      <c r="P38" s="47"/>
     </row>
     <row r="39" spans="1:16" ht="15" thickBot="1">
       <c r="A39" s="19">
@@ -3891,11 +3891,11 @@
       <c r="B39" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C39" s="48" t="s">
+      <c r="C39" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="D39" s="49"/>
-      <c r="E39" s="50"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="39"/>
       <c r="F39" s="9">
         <v>2</v>
       </c>
@@ -3905,11 +3905,11 @@
       <c r="H39" s="20" t="s">
         <v>242</v>
       </c>
-      <c r="L39" s="59"/>
-      <c r="M39" s="51"/>
-      <c r="N39" s="51"/>
-      <c r="O39" s="51"/>
-      <c r="P39" s="52"/>
+      <c r="L39" s="48"/>
+      <c r="M39" s="49"/>
+      <c r="N39" s="49"/>
+      <c r="O39" s="49"/>
+      <c r="P39" s="50"/>
     </row>
     <row r="40" spans="1:16" ht="15" thickBot="1">
       <c r="A40" s="19">
@@ -3918,11 +3918,11 @@
       <c r="B40" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C40" s="48" t="s">
+      <c r="C40" s="37" t="s">
         <v>89</v>
       </c>
-      <c r="D40" s="49"/>
-      <c r="E40" s="50"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="39"/>
       <c r="F40" s="9">
         <v>1</v>
       </c>
@@ -3940,11 +3940,11 @@
       <c r="B41" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C41" s="48" t="s">
+      <c r="C41" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="D41" s="49"/>
-      <c r="E41" s="50"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="39"/>
       <c r="F41" s="9">
         <v>1</v>
       </c>
@@ -3954,13 +3954,13 @@
       <c r="H41" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="L41" s="55" t="s">
+      <c r="L41" s="51" t="s">
         <v>91</v>
       </c>
-      <c r="M41" s="56"/>
-      <c r="N41" s="56"/>
-      <c r="O41" s="56"/>
-      <c r="P41" s="57"/>
+      <c r="M41" s="52"/>
+      <c r="N41" s="52"/>
+      <c r="O41" s="52"/>
+      <c r="P41" s="53"/>
     </row>
     <row r="42" spans="1:16">
       <c r="A42" s="19">
@@ -3969,11 +3969,11 @@
       <c r="B42" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="48" t="s">
+      <c r="C42" s="37" t="s">
         <v>92</v>
       </c>
-      <c r="D42" s="49"/>
-      <c r="E42" s="50"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="39"/>
       <c r="F42" s="9">
         <v>1</v>
       </c>
@@ -3983,13 +3983,13 @@
       <c r="H42" s="20" t="s">
         <v>227</v>
       </c>
-      <c r="L42" s="58" t="s">
+      <c r="L42" s="45" t="s">
         <v>230</v>
       </c>
-      <c r="M42" s="43"/>
-      <c r="N42" s="43"/>
-      <c r="O42" s="43"/>
-      <c r="P42" s="44"/>
+      <c r="M42" s="46"/>
+      <c r="N42" s="46"/>
+      <c r="O42" s="46"/>
+      <c r="P42" s="47"/>
     </row>
     <row r="43" spans="1:16" ht="15" thickBot="1">
       <c r="A43" s="19">
@@ -3998,11 +3998,11 @@
       <c r="B43" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C43" s="48" t="s">
+      <c r="C43" s="37" t="s">
         <v>93</v>
       </c>
-      <c r="D43" s="49"/>
-      <c r="E43" s="50"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="39"/>
       <c r="F43" s="9">
         <v>1</v>
       </c>
@@ -4012,11 +4012,11 @@
       <c r="H43" s="20" t="s">
         <v>244</v>
       </c>
-      <c r="L43" s="59"/>
-      <c r="M43" s="51"/>
-      <c r="N43" s="51"/>
-      <c r="O43" s="51"/>
-      <c r="P43" s="52"/>
+      <c r="L43" s="48"/>
+      <c r="M43" s="49"/>
+      <c r="N43" s="49"/>
+      <c r="O43" s="49"/>
+      <c r="P43" s="50"/>
     </row>
     <row r="44" spans="1:16" ht="15" thickBot="1">
       <c r="A44" s="17">
@@ -4025,11 +4025,11 @@
       <c r="B44" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C44" s="45" t="s">
+      <c r="C44" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="D44" s="46"/>
-      <c r="E44" s="47"/>
+      <c r="D44" s="35"/>
+      <c r="E44" s="36"/>
       <c r="F44" s="7">
         <v>1</v>
       </c>
@@ -4047,11 +4047,11 @@
       <c r="B45" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C45" s="45" t="s">
+      <c r="C45" s="34" t="s">
         <v>95</v>
       </c>
-      <c r="D45" s="46"/>
-      <c r="E45" s="47"/>
+      <c r="D45" s="35"/>
+      <c r="E45" s="36"/>
       <c r="F45" s="7">
         <v>2</v>
       </c>
@@ -4061,13 +4061,13 @@
       <c r="H45" s="18" t="s">
         <v>246</v>
       </c>
-      <c r="L45" s="55" t="s">
+      <c r="L45" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="M45" s="56"/>
-      <c r="N45" s="56"/>
-      <c r="O45" s="56"/>
-      <c r="P45" s="57"/>
+      <c r="M45" s="52"/>
+      <c r="N45" s="52"/>
+      <c r="O45" s="52"/>
+      <c r="P45" s="53"/>
     </row>
     <row r="46" spans="1:16">
       <c r="A46" s="17">
@@ -4076,11 +4076,11 @@
       <c r="B46" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C46" s="45" t="s">
+      <c r="C46" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="D46" s="46"/>
-      <c r="E46" s="47"/>
+      <c r="D46" s="35"/>
+      <c r="E46" s="36"/>
       <c r="F46" s="7">
         <v>1</v>
       </c>
@@ -4090,13 +4090,13 @@
       <c r="H46" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="L46" s="58" t="s">
+      <c r="L46" s="45" t="s">
         <v>266</v>
       </c>
-      <c r="M46" s="43"/>
-      <c r="N46" s="43"/>
-      <c r="O46" s="43"/>
-      <c r="P46" s="44"/>
+      <c r="M46" s="46"/>
+      <c r="N46" s="46"/>
+      <c r="O46" s="46"/>
+      <c r="P46" s="47"/>
     </row>
     <row r="47" spans="1:16" ht="15" thickBot="1">
       <c r="A47" s="17">
@@ -4105,11 +4105,11 @@
       <c r="B47" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C47" s="45" t="s">
+      <c r="C47" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="D47" s="46"/>
-      <c r="E47" s="47"/>
+      <c r="D47" s="35"/>
+      <c r="E47" s="36"/>
       <c r="F47" s="7">
         <v>1</v>
       </c>
@@ -4119,11 +4119,11 @@
       <c r="H47" s="18" t="s">
         <v>231</v>
       </c>
-      <c r="L47" s="59"/>
-      <c r="M47" s="51"/>
-      <c r="N47" s="51"/>
-      <c r="O47" s="51"/>
-      <c r="P47" s="52"/>
+      <c r="L47" s="48"/>
+      <c r="M47" s="49"/>
+      <c r="N47" s="49"/>
+      <c r="O47" s="49"/>
+      <c r="P47" s="50"/>
     </row>
     <row r="48" spans="1:16" ht="15" thickBot="1">
       <c r="A48" s="19">
@@ -4132,11 +4132,11 @@
       <c r="B48" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C48" s="48" t="s">
+      <c r="C48" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="D48" s="49"/>
-      <c r="E48" s="50"/>
+      <c r="D48" s="38"/>
+      <c r="E48" s="39"/>
       <c r="F48" s="9">
         <v>1</v>
       </c>
@@ -4154,11 +4154,11 @@
       <c r="B49" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C49" s="48" t="s">
+      <c r="C49" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="D49" s="49"/>
-      <c r="E49" s="50"/>
+      <c r="D49" s="38"/>
+      <c r="E49" s="39"/>
       <c r="F49" s="9" t="s">
         <v>196</v>
       </c>
@@ -4168,13 +4168,13 @@
       <c r="H49" s="20" t="s">
         <v>247</v>
       </c>
-      <c r="L49" s="55" t="s">
+      <c r="L49" s="51" t="s">
         <v>101</v>
       </c>
-      <c r="M49" s="56"/>
-      <c r="N49" s="56"/>
-      <c r="O49" s="56"/>
-      <c r="P49" s="57"/>
+      <c r="M49" s="52"/>
+      <c r="N49" s="52"/>
+      <c r="O49" s="52"/>
+      <c r="P49" s="53"/>
     </row>
     <row r="50" spans="1:16">
       <c r="A50" s="19">
@@ -4183,11 +4183,11 @@
       <c r="B50" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C50" s="48" t="s">
+      <c r="C50" s="37" t="s">
         <v>102</v>
       </c>
-      <c r="D50" s="49"/>
-      <c r="E50" s="50"/>
+      <c r="D50" s="38"/>
+      <c r="E50" s="39"/>
       <c r="F50" s="9">
         <v>1</v>
       </c>
@@ -4197,13 +4197,13 @@
       <c r="H50" s="20" t="s">
         <v>248</v>
       </c>
-      <c r="L50" s="58" t="s">
+      <c r="L50" s="45" t="s">
         <v>230</v>
       </c>
-      <c r="M50" s="43"/>
-      <c r="N50" s="43"/>
-      <c r="O50" s="43"/>
-      <c r="P50" s="44"/>
+      <c r="M50" s="46"/>
+      <c r="N50" s="46"/>
+      <c r="O50" s="46"/>
+      <c r="P50" s="47"/>
     </row>
     <row r="51" spans="1:16" ht="15" thickBot="1">
       <c r="A51" s="19">
@@ -4212,11 +4212,11 @@
       <c r="B51" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C51" s="48" t="s">
+      <c r="C51" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="D51" s="49"/>
-      <c r="E51" s="50"/>
+      <c r="D51" s="38"/>
+      <c r="E51" s="39"/>
       <c r="F51" s="9">
         <v>1</v>
       </c>
@@ -4226,11 +4226,11 @@
       <c r="H51" s="20" t="s">
         <v>249</v>
       </c>
-      <c r="L51" s="59"/>
-      <c r="M51" s="51"/>
-      <c r="N51" s="51"/>
-      <c r="O51" s="51"/>
-      <c r="P51" s="52"/>
+      <c r="L51" s="48"/>
+      <c r="M51" s="49"/>
+      <c r="N51" s="49"/>
+      <c r="O51" s="49"/>
+      <c r="P51" s="50"/>
     </row>
     <row r="52" spans="1:16">
       <c r="A52" s="17">
@@ -4239,11 +4239,11 @@
       <c r="B52" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C52" s="45" t="s">
+      <c r="C52" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="D52" s="46"/>
-      <c r="E52" s="47"/>
+      <c r="D52" s="35"/>
+      <c r="E52" s="36"/>
       <c r="F52" s="7">
         <v>1</v>
       </c>
@@ -4261,11 +4261,11 @@
       <c r="B53" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C53" s="45" t="s">
+      <c r="C53" s="34" t="s">
         <v>105</v>
       </c>
-      <c r="D53" s="46"/>
-      <c r="E53" s="47"/>
+      <c r="D53" s="35"/>
+      <c r="E53" s="36"/>
       <c r="F53" s="7">
         <v>2</v>
       </c>
@@ -4273,7 +4273,7 @@
         <v>200</v>
       </c>
       <c r="H53" s="18" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="54" spans="1:16">
@@ -4283,11 +4283,11 @@
       <c r="B54" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C54" s="45" t="s">
+      <c r="C54" s="34" t="s">
         <v>106</v>
       </c>
-      <c r="D54" s="46"/>
-      <c r="E54" s="47"/>
+      <c r="D54" s="35"/>
+      <c r="E54" s="36"/>
       <c r="F54" s="7">
         <v>1</v>
       </c>
@@ -4305,11 +4305,11 @@
       <c r="B55" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C55" s="45" t="s">
+      <c r="C55" s="34" t="s">
         <v>107</v>
       </c>
-      <c r="D55" s="46"/>
-      <c r="E55" s="47"/>
+      <c r="D55" s="35"/>
+      <c r="E55" s="36"/>
       <c r="F55" s="7">
         <v>1</v>
       </c>
@@ -4327,11 +4327,11 @@
       <c r="B56" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C56" s="48" t="s">
+      <c r="C56" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="D56" s="49"/>
-      <c r="E56" s="50"/>
+      <c r="D56" s="38"/>
+      <c r="E56" s="39"/>
       <c r="F56" s="9">
         <v>2</v>
       </c>
@@ -4349,11 +4349,11 @@
       <c r="B57" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C57" s="48" t="s">
+      <c r="C57" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="D57" s="49"/>
-      <c r="E57" s="50"/>
+      <c r="D57" s="38"/>
+      <c r="E57" s="39"/>
       <c r="F57" s="9">
         <v>1</v>
       </c>
@@ -4365,14 +4365,14 @@
       </c>
     </row>
     <row r="58" spans="1:16">
-      <c r="A58" s="66"/>
-      <c r="B58" s="67"/>
-      <c r="C58" s="67"/>
-      <c r="D58" s="67"/>
-      <c r="E58" s="67"/>
-      <c r="F58" s="67"/>
-      <c r="G58" s="67"/>
-      <c r="H58" s="68"/>
+      <c r="A58" s="54"/>
+      <c r="B58" s="55"/>
+      <c r="C58" s="55"/>
+      <c r="D58" s="55"/>
+      <c r="E58" s="55"/>
+      <c r="F58" s="55"/>
+      <c r="G58" s="55"/>
+      <c r="H58" s="56"/>
     </row>
     <row r="59" spans="1:16">
       <c r="A59" s="19">
@@ -4381,11 +4381,11 @@
       <c r="B59" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C59" s="48" t="s">
+      <c r="C59" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="D59" s="49"/>
-      <c r="E59" s="50"/>
+      <c r="D59" s="38"/>
+      <c r="E59" s="39"/>
       <c r="F59" s="9">
         <v>1</v>
       </c>
@@ -4403,11 +4403,11 @@
       <c r="B60" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C60" s="48" t="s">
+      <c r="C60" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="D60" s="49"/>
-      <c r="E60" s="50"/>
+      <c r="D60" s="38"/>
+      <c r="E60" s="39"/>
       <c r="F60" s="9">
         <v>1</v>
       </c>
@@ -4425,11 +4425,11 @@
       <c r="B61" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C61" s="45" t="s">
+      <c r="C61" s="34" t="s">
         <v>112</v>
       </c>
-      <c r="D61" s="46"/>
-      <c r="E61" s="47"/>
+      <c r="D61" s="35"/>
+      <c r="E61" s="36"/>
       <c r="F61" s="7">
         <v>2</v>
       </c>
@@ -4447,11 +4447,11 @@
       <c r="B62" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C62" s="45" t="s">
+      <c r="C62" s="34" t="s">
         <v>113</v>
       </c>
-      <c r="D62" s="46"/>
-      <c r="E62" s="47"/>
+      <c r="D62" s="35"/>
+      <c r="E62" s="36"/>
       <c r="F62" s="7">
         <v>1</v>
       </c>
@@ -4469,11 +4469,11 @@
       <c r="B63" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C63" s="45" t="s">
+      <c r="C63" s="34" t="s">
         <v>114</v>
       </c>
-      <c r="D63" s="46"/>
-      <c r="E63" s="47"/>
+      <c r="D63" s="35"/>
+      <c r="E63" s="36"/>
       <c r="F63" s="7" t="s">
         <v>196</v>
       </c>
@@ -4491,11 +4491,11 @@
       <c r="B64" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C64" s="45" t="s">
+      <c r="C64" s="34" t="s">
         <v>115</v>
       </c>
-      <c r="D64" s="46"/>
-      <c r="E64" s="47"/>
+      <c r="D64" s="35"/>
+      <c r="E64" s="36"/>
       <c r="F64" s="7" t="s">
         <v>196</v>
       </c>
@@ -4513,11 +4513,11 @@
       <c r="B65" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C65" s="45" t="s">
+      <c r="C65" s="34" t="s">
         <v>116</v>
       </c>
-      <c r="D65" s="46"/>
-      <c r="E65" s="47"/>
+      <c r="D65" s="35"/>
+      <c r="E65" s="36"/>
       <c r="F65" s="7">
         <v>2</v>
       </c>
@@ -4535,11 +4535,11 @@
       <c r="B66" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C66" s="45" t="s">
+      <c r="C66" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="D66" s="46"/>
-      <c r="E66" s="47"/>
+      <c r="D66" s="35"/>
+      <c r="E66" s="36"/>
       <c r="F66" s="8">
         <v>2</v>
       </c>
@@ -4557,11 +4557,11 @@
       <c r="B67" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C67" s="48" t="s">
+      <c r="C67" s="37" t="s">
         <v>118</v>
       </c>
-      <c r="D67" s="49"/>
-      <c r="E67" s="50"/>
+      <c r="D67" s="38"/>
+      <c r="E67" s="39"/>
       <c r="F67" s="9">
         <v>2</v>
       </c>
@@ -4579,11 +4579,11 @@
       <c r="B68" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C68" s="48" t="s">
+      <c r="C68" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="D68" s="49"/>
-      <c r="E68" s="50"/>
+      <c r="D68" s="38"/>
+      <c r="E68" s="39"/>
       <c r="F68" s="9">
         <v>1</v>
       </c>
@@ -4601,11 +4601,11 @@
       <c r="B69" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C69" s="48" t="s">
+      <c r="C69" s="37" t="s">
         <v>120</v>
       </c>
-      <c r="D69" s="49"/>
-      <c r="E69" s="50"/>
+      <c r="D69" s="38"/>
+      <c r="E69" s="39"/>
       <c r="F69" s="9">
         <v>1</v>
       </c>
@@ -4623,11 +4623,11 @@
       <c r="B70" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C70" s="48" t="s">
+      <c r="C70" s="37" t="s">
         <v>121</v>
       </c>
-      <c r="D70" s="49"/>
-      <c r="E70" s="50"/>
+      <c r="D70" s="38"/>
+      <c r="E70" s="39"/>
       <c r="F70" s="9">
         <v>1</v>
       </c>
@@ -4645,11 +4645,11 @@
       <c r="B71" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C71" s="48" t="s">
+      <c r="C71" s="37" t="s">
         <v>122</v>
       </c>
-      <c r="D71" s="49"/>
-      <c r="E71" s="50"/>
+      <c r="D71" s="38"/>
+      <c r="E71" s="39"/>
       <c r="F71" s="9">
         <v>2</v>
       </c>
@@ -4667,11 +4667,11 @@
       <c r="B72" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C72" s="48" t="s">
+      <c r="C72" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="D72" s="49"/>
-      <c r="E72" s="50"/>
+      <c r="D72" s="38"/>
+      <c r="E72" s="39"/>
       <c r="F72" s="9">
         <v>1</v>
       </c>
@@ -4689,11 +4689,11 @@
       <c r="B73" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C73" s="45" t="s">
+      <c r="C73" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="D73" s="46"/>
-      <c r="E73" s="47"/>
+      <c r="D73" s="35"/>
+      <c r="E73" s="36"/>
       <c r="F73" s="7">
         <v>1</v>
       </c>
@@ -4711,11 +4711,11 @@
       <c r="B74" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C74" s="45" t="s">
+      <c r="C74" s="34" t="s">
         <v>125</v>
       </c>
-      <c r="D74" s="46"/>
-      <c r="E74" s="47"/>
+      <c r="D74" s="35"/>
+      <c r="E74" s="36"/>
       <c r="F74" s="7">
         <v>2</v>
       </c>
@@ -4733,11 +4733,11 @@
       <c r="B75" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C75" s="45" t="s">
+      <c r="C75" s="34" t="s">
         <v>126</v>
       </c>
-      <c r="D75" s="46"/>
-      <c r="E75" s="47"/>
+      <c r="D75" s="35"/>
+      <c r="E75" s="36"/>
       <c r="F75" s="2">
         <v>1</v>
       </c>
@@ -4755,11 +4755,11 @@
       <c r="B76" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C76" s="45" t="s">
+      <c r="C76" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="D76" s="46"/>
-      <c r="E76" s="47"/>
+      <c r="D76" s="35"/>
+      <c r="E76" s="36"/>
       <c r="F76" s="2">
         <v>2</v>
       </c>
@@ -4777,11 +4777,11 @@
       <c r="B77" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C77" s="45" t="s">
+      <c r="C77" s="34" t="s">
         <v>128</v>
       </c>
-      <c r="D77" s="46"/>
-      <c r="E77" s="47"/>
+      <c r="D77" s="35"/>
+      <c r="E77" s="36"/>
       <c r="F77" s="7">
         <v>2</v>
       </c>
@@ -4799,15 +4799,15 @@
       <c r="B78" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C78" s="45" t="s">
+      <c r="C78" s="34" t="s">
         <v>129</v>
       </c>
-      <c r="D78" s="46"/>
-      <c r="E78" s="47"/>
+      <c r="D78" s="35"/>
+      <c r="E78" s="36"/>
       <c r="F78" s="7">
         <v>1</v>
       </c>
-      <c r="G78" s="95" t="s">
+      <c r="G78" s="33" t="s">
         <v>199</v>
       </c>
       <c r="H78" s="18" t="s">
@@ -4821,11 +4821,11 @@
       <c r="B79" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C79" s="48" t="s">
+      <c r="C79" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="D79" s="49"/>
-      <c r="E79" s="50"/>
+      <c r="D79" s="38"/>
+      <c r="E79" s="39"/>
       <c r="F79" s="9">
         <v>1</v>
       </c>
@@ -4843,11 +4843,11 @@
       <c r="B80" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C80" s="48" t="s">
+      <c r="C80" s="37" t="s">
         <v>131</v>
       </c>
-      <c r="D80" s="49"/>
-      <c r="E80" s="50"/>
+      <c r="D80" s="38"/>
+      <c r="E80" s="39"/>
       <c r="F80" s="9">
         <v>1</v>
       </c>
@@ -4865,11 +4865,11 @@
       <c r="B81" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C81" s="48" t="s">
+      <c r="C81" s="37" t="s">
         <v>132</v>
       </c>
-      <c r="D81" s="49"/>
-      <c r="E81" s="50"/>
+      <c r="D81" s="38"/>
+      <c r="E81" s="39"/>
       <c r="F81" s="9">
         <v>2</v>
       </c>
@@ -4887,11 +4887,11 @@
       <c r="B82" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="C82" s="71" t="s">
+      <c r="C82" s="40" t="s">
         <v>133</v>
       </c>
-      <c r="D82" s="72"/>
-      <c r="E82" s="73"/>
+      <c r="D82" s="41"/>
+      <c r="E82" s="42"/>
       <c r="F82" s="23">
         <v>1</v>
       </c>
@@ -4899,34 +4899,103 @@
         <v>220</v>
       </c>
       <c r="H82" s="24" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="139">
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="C79:E79"/>
-    <mergeCell ref="C80:E80"/>
-    <mergeCell ref="C81:E81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="C74:E74"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="C77:E77"/>
-    <mergeCell ref="C66:E66"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="C71:E71"/>
-    <mergeCell ref="C60:E60"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="A5:T6"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="J8:Q8"/>
+    <mergeCell ref="J7:Q7"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="O16:Q16"/>
+    <mergeCell ref="L10:N10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="O11:Q11"/>
+    <mergeCell ref="L12:N12"/>
+    <mergeCell ref="O12:Q12"/>
+    <mergeCell ref="L13:N13"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="O9:Q9"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="O17:Q17"/>
+    <mergeCell ref="L18:N18"/>
+    <mergeCell ref="O18:Q18"/>
+    <mergeCell ref="O13:Q13"/>
+    <mergeCell ref="L14:N14"/>
+    <mergeCell ref="O14:Q14"/>
+    <mergeCell ref="L15:N15"/>
+    <mergeCell ref="O15:Q15"/>
+    <mergeCell ref="L16:N16"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="L20:N20"/>
+    <mergeCell ref="O20:Q20"/>
+    <mergeCell ref="L21:N21"/>
+    <mergeCell ref="O21:Q21"/>
+    <mergeCell ref="L19:N19"/>
+    <mergeCell ref="O19:Q19"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="L23:P23"/>
+    <mergeCell ref="L24:P25"/>
+    <mergeCell ref="L27:P27"/>
+    <mergeCell ref="L28:L29"/>
+    <mergeCell ref="L30:L31"/>
+    <mergeCell ref="M28:P29"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="M30:P31"/>
+    <mergeCell ref="L33:P33"/>
+    <mergeCell ref="L34:P35"/>
+    <mergeCell ref="L37:P37"/>
+    <mergeCell ref="L38:P39"/>
+    <mergeCell ref="L41:P41"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="L42:P43"/>
+    <mergeCell ref="L45:P45"/>
+    <mergeCell ref="L46:P47"/>
+    <mergeCell ref="L49:P49"/>
+    <mergeCell ref="L50:P51"/>
+    <mergeCell ref="A58:H58"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C2:F2"/>
@@ -4951,98 +5020,29 @@
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="C25:E25"/>
     <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="C54:E54"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="C57:E57"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="L42:P43"/>
-    <mergeCell ref="L45:P45"/>
-    <mergeCell ref="L46:P47"/>
-    <mergeCell ref="L49:P49"/>
-    <mergeCell ref="L50:P51"/>
-    <mergeCell ref="A58:H58"/>
-    <mergeCell ref="L33:P33"/>
-    <mergeCell ref="L34:P35"/>
-    <mergeCell ref="L37:P37"/>
-    <mergeCell ref="L38:P39"/>
-    <mergeCell ref="L41:P41"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="A33:H33"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="L23:P23"/>
-    <mergeCell ref="L24:P25"/>
-    <mergeCell ref="L27:P27"/>
-    <mergeCell ref="L28:L29"/>
-    <mergeCell ref="L30:L31"/>
-    <mergeCell ref="M28:P29"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="M30:P31"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="L20:N20"/>
-    <mergeCell ref="O20:Q20"/>
-    <mergeCell ref="L21:N21"/>
-    <mergeCell ref="O21:Q21"/>
-    <mergeCell ref="L19:N19"/>
-    <mergeCell ref="O19:Q19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="L17:N17"/>
-    <mergeCell ref="O17:Q17"/>
-    <mergeCell ref="L18:N18"/>
-    <mergeCell ref="O18:Q18"/>
-    <mergeCell ref="O13:Q13"/>
-    <mergeCell ref="L14:N14"/>
-    <mergeCell ref="O14:Q14"/>
-    <mergeCell ref="L15:N15"/>
-    <mergeCell ref="O15:Q15"/>
-    <mergeCell ref="L16:N16"/>
-    <mergeCell ref="A5:T6"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="J8:Q8"/>
-    <mergeCell ref="J7:Q7"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="O16:Q16"/>
-    <mergeCell ref="L10:N10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="L11:N11"/>
-    <mergeCell ref="O11:Q11"/>
-    <mergeCell ref="L12:N12"/>
-    <mergeCell ref="O12:Q12"/>
-    <mergeCell ref="L13:N13"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:N9"/>
-    <mergeCell ref="O9:Q9"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="C66:E66"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="C80:E80"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="C74:E74"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="C77:E77"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>

</xml_diff>